<commit_message>
Fold data protection into Compliance Monitoring Pack and financial promotions into Consumer Duty Pack
Removes the two proposed new packs so every document sits in an existing
Stripe product with unchanged prices and payment links.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0185GJD35Lj4maZQfYQD6Tsw
</commit_message>
<xml_diff>
--- a/framework-templates/Document_Log_Pricing_v2.0.xlsx
+++ b/framework-templates/Document_Log_Pricing_v2.0.xlsx
@@ -58,7 +58,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -69,11 +69,6 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.3999755851924192"/>
         <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -121,7 +116,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -169,19 +164,16 @@
     <xf numFmtId="165" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1042,7 +1034,7 @@
       </c>
       <c r="N14" s="13" t="inlineStr">
         <is>
-          <t>Compliance Monitoring Pack; Customer Due Diligence Pack; Consumer Duty Pack; Financial Promotions Pack</t>
+          <t>Compliance Monitoring Pack; Customer Due Diligence Pack; Consumer Duty Pack</t>
         </is>
       </c>
     </row>
@@ -1089,7 +1081,7 @@
       </c>
       <c r="N15" s="13" t="inlineStr">
         <is>
-          <t>AML Pack; Compliance Monitoring Pack; Risk Management Pack; Training Pack; Data Protection Pack</t>
+          <t>AML Pack; Compliance Monitoring Pack; Risk Management Pack; Training Pack</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1220,7 @@
       </c>
       <c r="N18" s="13" t="inlineStr">
         <is>
-          <t>Training Pack; Financial Promotions Pack</t>
+          <t>Training Pack; Consumer Duty Pack</t>
         </is>
       </c>
     </row>
@@ -1368,22 +1360,16 @@
     <row r="22">
       <c r="B22" s="13" t="inlineStr">
         <is>
-          <t>Customer Due Diligence Policy</t>
+          <t>Data Processing Policy</t>
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
         <is>
-          <t>Customer Due Diligence Pack</t>
-        </is>
-      </c>
-      <c r="D22" s="14" t="n">
-        <v>45</v>
-      </c>
-      <c r="E22" s="18" t="inlineStr">
-        <is>
-          <t>https://buy.stripe.com/28E4gs9xb4pv6OdeGDfbq00</t>
-        </is>
-      </c>
+          <t>Compliance Monitoring Pack</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="n"/>
+      <c r="E22" s="13" t="n"/>
       <c r="F22" s="13" t="n"/>
       <c r="G22" s="13" t="inlineStr">
         <is>
@@ -1409,7 +1395,7 @@
       </c>
       <c r="M22" s="13" t="inlineStr">
         <is>
-          <t>Customer_Due_Diligence_Policy_v2.0_Template.docx</t>
+          <t>Data_Processing_Policy_v2.0_Template.docx</t>
         </is>
       </c>
       <c r="N22" s="13" t="n"/>
@@ -1417,12 +1403,12 @@
     <row r="23">
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t>Customer Vulnerability Policy</t>
+          <t>Record of Processing Activities</t>
         </is>
       </c>
       <c r="C23" s="13" t="inlineStr">
         <is>
-          <t>Customer Due Diligence Pack</t>
+          <t>Compliance Monitoring Pack</t>
         </is>
       </c>
       <c r="D23" s="13" t="n"/>
@@ -1447,25 +1433,29 @@
       </c>
       <c r="L23" s="13" t="inlineStr">
         <is>
-          <t>Policy.</t>
+          <t>Register.</t>
         </is>
       </c>
       <c r="M23" s="13" t="inlineStr">
         <is>
-          <t>Customer_Vulnerability_Policy_v2.0_Template.docx</t>
-        </is>
-      </c>
-      <c r="N23" s="13" t="n"/>
+          <t>Record_of_Processing_Activities_v2.0_Template.xlsx</t>
+        </is>
+      </c>
+      <c r="N23" s="13" t="inlineStr">
+        <is>
+          <t>Customer Due Diligence Pack</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="B24" s="13" t="inlineStr">
         <is>
-          <t>Customer Due Diligence Checklist</t>
+          <t>Data Rights Request Log</t>
         </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
-          <t>Customer Due Diligence Pack</t>
+          <t>Compliance Monitoring Pack</t>
         </is>
       </c>
       <c r="D24" s="13" t="n"/>
@@ -1495,24 +1485,20 @@
       </c>
       <c r="M24" s="13" t="inlineStr">
         <is>
-          <t>Customer_Due_Diligence_Checklist_v2.0_Template.xlsx</t>
-        </is>
-      </c>
-      <c r="N24" s="13" t="inlineStr">
-        <is>
-          <t>AML Pack</t>
-        </is>
-      </c>
+          <t>Data_Rights_Request_Log_v2.0_Template.xlsx</t>
+        </is>
+      </c>
+      <c r="N24" s="13" t="n"/>
     </row>
     <row r="25">
       <c r="B25" s="13" t="inlineStr">
         <is>
-          <t>Enhanced Due Diligence Checklist</t>
+          <t>Data Breach Log</t>
         </is>
       </c>
       <c r="C25" s="13" t="inlineStr">
         <is>
-          <t>Customer Due Diligence Pack</t>
+          <t>Compliance Monitoring Pack</t>
         </is>
       </c>
       <c r="D25" s="13" t="n"/>
@@ -1542,24 +1528,20 @@
       </c>
       <c r="M25" s="13" t="inlineStr">
         <is>
-          <t>Enhanced_Due_Diligence_Checklist_v2.0_Template.xlsx</t>
-        </is>
-      </c>
-      <c r="N25" s="13" t="inlineStr">
-        <is>
-          <t>AML Pack</t>
-        </is>
-      </c>
+          <t>Data_Breach_Log_v2.0_Template.xlsx</t>
+        </is>
+      </c>
+      <c r="N25" s="13" t="n"/>
     </row>
     <row r="26">
       <c r="B26" s="13" t="inlineStr">
         <is>
-          <t>Customer Due Diligence Register</t>
+          <t>Data Protection Complaints Log</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>Customer Due Diligence Pack</t>
+          <t>Compliance Monitoring Pack</t>
         </is>
       </c>
       <c r="D26" s="13" t="n"/>
@@ -1589,34 +1571,28 @@
       </c>
       <c r="M26" s="13" t="inlineStr">
         <is>
-          <t>Customer_Due_Diligence_Register_v2.0_Template.xlsx</t>
+          <t>Data_Protection_Complaints_Log_v2.0_Template.xlsx</t>
         </is>
       </c>
       <c r="N26" s="13" t="inlineStr">
         <is>
-          <t>AML Pack; Compliance Monitoring Pack</t>
+          <t>Complaints Pack</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="13" t="inlineStr">
         <is>
-          <t>SM&amp;CR Statement of Responsibilities</t>
+          <t>Data Retention Schedule</t>
         </is>
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>Senior Management Pack</t>
-        </is>
-      </c>
-      <c r="D27" s="14" t="n">
-        <v>35</v>
-      </c>
-      <c r="E27" s="18" t="inlineStr">
-        <is>
-          <t>https://buy.stripe.com/4gMdR238NbRX2xXcyvfbq04</t>
-        </is>
-      </c>
+          <t>Compliance Monitoring Pack</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="n"/>
+      <c r="E27" s="13" t="n"/>
       <c r="F27" s="13" t="n"/>
       <c r="G27" s="13" t="inlineStr">
         <is>
@@ -1637,12 +1613,12 @@
       </c>
       <c r="L27" s="13" t="inlineStr">
         <is>
-          <t>Policy.</t>
+          <t>Register.</t>
         </is>
       </c>
       <c r="M27" s="13" t="inlineStr">
         <is>
-          <t>SMCR_Statement_of_Responsibilities_v2.0_Template.docx</t>
+          <t>Data_Retention_Schedule_v2.0_Template.xlsx</t>
         </is>
       </c>
       <c r="N27" s="13" t="n"/>
@@ -1650,12 +1626,12 @@
     <row r="28">
       <c r="B28" s="13" t="inlineStr">
         <is>
-          <t>FIT and Proper Questionnaire</t>
+          <t>DPIA Register</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>Senior Management Pack</t>
+          <t>Compliance Monitoring Pack</t>
         </is>
       </c>
       <c r="D28" s="13" t="n"/>
@@ -1663,21 +1639,29 @@
       <c r="F28" s="13" t="n"/>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="H28" s="13" t="n"/>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="H28" s="13" t="inlineStr">
+        <is>
+          <t>KMS Compliance (AI-assisted v2.0 rewrite)</t>
+        </is>
+      </c>
       <c r="I28" s="13" t="n"/>
-      <c r="J28" s="16" t="n"/>
-      <c r="K28" s="16" t="n"/>
+      <c r="J28" s="16" t="n">
+        <v>46290</v>
+      </c>
+      <c r="K28" s="16" t="n">
+        <v>46655</v>
+      </c>
       <c r="L28" s="13" t="inlineStr">
         <is>
-          <t>Form. Not updated in the v2.0 rewrite – review separately.</t>
+          <t>Register.</t>
         </is>
       </c>
       <c r="M28" s="13" t="inlineStr">
         <is>
-          <t>FIT_and_Proper_Questionnaire_v1.0.docx</t>
+          <t>DPIA_Register_v2.0_Template.xlsx</t>
         </is>
       </c>
       <c r="N28" s="13" t="n"/>
@@ -1685,20 +1669,20 @@
     <row r="29">
       <c r="B29" s="13" t="inlineStr">
         <is>
-          <t>Consumer Duty Implementation and Embedding Plan</t>
+          <t>Customer Due Diligence Policy</t>
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr">
         <is>
-          <t>Consumer Duty Pack</t>
+          <t>Customer Due Diligence Pack</t>
         </is>
       </c>
       <c r="D29" s="14" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="E29" s="18" t="inlineStr">
         <is>
-          <t>https://buy.stripe.com/28E28kbFj1djb4t41Zfbq06</t>
+          <t>https://buy.stripe.com/28E4gs9xb4pv6OdeGDfbq00</t>
         </is>
       </c>
       <c r="F29" s="13" t="n"/>
@@ -1726,7 +1710,7 @@
       </c>
       <c r="M29" s="13" t="inlineStr">
         <is>
-          <t>Consumer_Duty_Implementation_Plan_v2.0_Template.docx</t>
+          <t>Customer_Due_Diligence_Policy_v2.0_Template.docx</t>
         </is>
       </c>
       <c r="N29" s="13" t="n"/>
@@ -1734,12 +1718,12 @@
     <row r="30">
       <c r="B30" s="13" t="inlineStr">
         <is>
-          <t>Consumer Duty Outcome MI</t>
+          <t>Customer Vulnerability Policy</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>Consumer Duty Pack</t>
+          <t>Customer Due Diligence Pack</t>
         </is>
       </c>
       <c r="D30" s="13" t="n"/>
@@ -1764,29 +1748,25 @@
       </c>
       <c r="L30" s="13" t="inlineStr">
         <is>
-          <t>Register.</t>
+          <t>Policy.</t>
         </is>
       </c>
       <c r="M30" s="13" t="inlineStr">
         <is>
-          <t>Consumer_Duty_Outcome_MI_v2.0_Template.xlsx</t>
-        </is>
-      </c>
-      <c r="N30" s="13" t="inlineStr">
-        <is>
-          <t>Complaints Pack; Compliance Monitoring Pack; Customer Due Diligence Pack; Risk Management Pack</t>
-        </is>
-      </c>
+          <t>Customer_Vulnerability_Policy_v2.0_Template.docx</t>
+        </is>
+      </c>
+      <c r="N30" s="13" t="n"/>
     </row>
     <row r="31">
       <c r="B31" s="13" t="inlineStr">
         <is>
-          <t>Target Market Register</t>
+          <t>Customer Due Diligence Checklist</t>
         </is>
       </c>
       <c r="C31" s="13" t="inlineStr">
         <is>
-          <t>Consumer Duty Pack</t>
+          <t>Customer Due Diligence Pack</t>
         </is>
       </c>
       <c r="D31" s="13" t="n"/>
@@ -1816,20 +1796,24 @@
       </c>
       <c r="M31" s="13" t="inlineStr">
         <is>
-          <t>Target_Market_Register_v2.0_Template.xlsx</t>
-        </is>
-      </c>
-      <c r="N31" s="13" t="n"/>
+          <t>Customer_Due_Diligence_Checklist_v2.0_Template.xlsx</t>
+        </is>
+      </c>
+      <c r="N31" s="13" t="inlineStr">
+        <is>
+          <t>AML Pack</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="B32" s="13" t="inlineStr">
         <is>
-          <t>Fair Value Register</t>
+          <t>Enhanced Due Diligence Checklist</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
         <is>
-          <t>Consumer Duty Pack</t>
+          <t>Customer Due Diligence Pack</t>
         </is>
       </c>
       <c r="D32" s="13" t="n"/>
@@ -1859,20 +1843,24 @@
       </c>
       <c r="M32" s="13" t="inlineStr">
         <is>
-          <t>Fair_Value_Register_v2.0_Template.xlsx</t>
-        </is>
-      </c>
-      <c r="N32" s="13" t="n"/>
+          <t>Enhanced_Due_Diligence_Checklist_v2.0_Template.xlsx</t>
+        </is>
+      </c>
+      <c r="N32" s="13" t="inlineStr">
+        <is>
+          <t>AML Pack</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="B33" s="13" t="inlineStr">
         <is>
-          <t>Consumer Duty Board Report Actions</t>
+          <t>Customer Due Diligence Register</t>
         </is>
       </c>
       <c r="C33" s="13" t="inlineStr">
         <is>
-          <t>Consumer Duty Pack</t>
+          <t>Customer Due Diligence Pack</t>
         </is>
       </c>
       <c r="D33" s="13" t="n"/>
@@ -1902,20 +1890,24 @@
       </c>
       <c r="M33" s="13" t="inlineStr">
         <is>
-          <t>Consumer_Duty_Board_Report_Actions_v2.0_Template.xlsx</t>
-        </is>
-      </c>
-      <c r="N33" s="13" t="n"/>
+          <t>Customer_Due_Diligence_Register_v2.0_Template.xlsx</t>
+        </is>
+      </c>
+      <c r="N33" s="13" t="inlineStr">
+        <is>
+          <t>AML Pack; Compliance Monitoring Pack</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="B34" s="13" t="inlineStr">
         <is>
-          <t>Risk Management Framework</t>
+          <t>SM&amp;CR Statement of Responsibilities</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
         <is>
-          <t>Risk Management Pack</t>
+          <t>Senior Management Pack</t>
         </is>
       </c>
       <c r="D34" s="14" t="n">
@@ -1923,7 +1915,7 @@
       </c>
       <c r="E34" s="18" t="inlineStr">
         <is>
-          <t>https://buy.stripe.com/7sY14g9xb5tz8Wl41Zfbq07</t>
+          <t>https://buy.stripe.com/4gMdR238NbRX2xXcyvfbq04</t>
         </is>
       </c>
       <c r="F34" s="13" t="n"/>
@@ -1951,7 +1943,7 @@
       </c>
       <c r="M34" s="13" t="inlineStr">
         <is>
-          <t>Risk_Management_Framework_v2.0_Template.docx</t>
+          <t>SMCR_Statement_of_Responsibilities_v2.0_Template.docx</t>
         </is>
       </c>
       <c r="N34" s="13" t="n"/>
@@ -1959,12 +1951,12 @@
     <row r="35">
       <c r="B35" s="13" t="inlineStr">
         <is>
-          <t>Risk Assessment Log</t>
+          <t>FIT and Proper Questionnaire</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
         <is>
-          <t>Risk Management Pack</t>
+          <t>Senior Management Pack</t>
         </is>
       </c>
       <c r="D35" s="13" t="n"/>
@@ -1972,46 +1964,34 @@
       <c r="F35" s="13" t="n"/>
       <c r="G35" s="13" t="inlineStr">
         <is>
-          <t>2.0</t>
-        </is>
-      </c>
-      <c r="H35" s="13" t="inlineStr">
-        <is>
-          <t>KMS Compliance (AI-assisted v2.0 rewrite)</t>
-        </is>
-      </c>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="H35" s="13" t="n"/>
       <c r="I35" s="13" t="n"/>
-      <c r="J35" s="16" t="n">
-        <v>46290</v>
-      </c>
-      <c r="K35" s="16" t="n">
-        <v>46655</v>
-      </c>
+      <c r="J35" s="16" t="n"/>
+      <c r="K35" s="16" t="n"/>
       <c r="L35" s="13" t="inlineStr">
         <is>
-          <t>Register.</t>
+          <t>Form. Not updated in the v2.0 rewrite – review separately.</t>
         </is>
       </c>
       <c r="M35" s="13" t="inlineStr">
         <is>
-          <t>Risk_Assessment_Log_v2.0_Template.xlsx</t>
-        </is>
-      </c>
-      <c r="N35" s="13" t="inlineStr">
-        <is>
-          <t>Compliance Monitoring Pack; Consumer Duty Pack</t>
-        </is>
-      </c>
+          <t>FIT_and_Proper_Questionnaire_v1.0.docx</t>
+        </is>
+      </c>
+      <c r="N35" s="13" t="n"/>
     </row>
     <row r="36">
       <c r="B36" s="13" t="inlineStr">
         <is>
-          <t>Training and Competence Policy</t>
+          <t>Consumer Duty Implementation and Embedding Plan</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>Training Pack</t>
+          <t>Consumer Duty Pack</t>
         </is>
       </c>
       <c r="D36" s="14" t="n">
@@ -2019,7 +1999,7 @@
       </c>
       <c r="E36" s="18" t="inlineStr">
         <is>
-          <t>https://buy.stripe.com/eVq28kaBf09fa0p6a7fbq08</t>
+          <t>https://buy.stripe.com/28E28kbFj1djb4t41Zfbq06</t>
         </is>
       </c>
       <c r="F36" s="13" t="n"/>
@@ -2047,7 +2027,7 @@
       </c>
       <c r="M36" s="13" t="inlineStr">
         <is>
-          <t>Training_and_Competence_Policy_v2.0_Template.docx</t>
+          <t>Consumer_Duty_Implementation_Plan_v2.0_Template.docx</t>
         </is>
       </c>
       <c r="N36" s="13" t="n"/>
@@ -2055,12 +2035,12 @@
     <row r="37">
       <c r="B37" s="13" t="inlineStr">
         <is>
-          <t>Training Matrix</t>
+          <t>Consumer Duty Outcome MI</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>Training Pack</t>
+          <t>Consumer Duty Pack</t>
         </is>
       </c>
       <c r="D37" s="13" t="n"/>
@@ -2090,20 +2070,24 @@
       </c>
       <c r="M37" s="13" t="inlineStr">
         <is>
-          <t>Training_Matrix_v2.0_Template.xlsx</t>
-        </is>
-      </c>
-      <c r="N37" s="13" t="n"/>
+          <t>Consumer_Duty_Outcome_MI_v2.0_Template.xlsx</t>
+        </is>
+      </c>
+      <c r="N37" s="13" t="inlineStr">
+        <is>
+          <t>Complaints Pack; Compliance Monitoring Pack; Customer Due Diligence Pack; Risk Management Pack</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="B38" s="13" t="inlineStr">
         <is>
-          <t>Training Log</t>
+          <t>Target Market Register</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>Training Pack</t>
+          <t>Consumer Duty Pack</t>
         </is>
       </c>
       <c r="D38" s="13" t="n"/>
@@ -2133,24 +2117,20 @@
       </c>
       <c r="M38" s="13" t="inlineStr">
         <is>
-          <t>Training_Log_v2.0_Template.xlsx</t>
-        </is>
-      </c>
-      <c r="N38" s="13" t="inlineStr">
-        <is>
-          <t>All other packs</t>
-        </is>
-      </c>
+          <t>Target_Market_Register_v2.0_Template.xlsx</t>
+        </is>
+      </c>
+      <c r="N38" s="13" t="n"/>
     </row>
     <row r="39">
       <c r="B39" s="13" t="inlineStr">
         <is>
-          <t>Competence Register</t>
+          <t>Fair Value Register</t>
         </is>
       </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
-          <t>Training Pack</t>
+          <t>Consumer Duty Pack</t>
         </is>
       </c>
       <c r="D39" s="13" t="n"/>
@@ -2180,24 +2160,20 @@
       </c>
       <c r="M39" s="13" t="inlineStr">
         <is>
-          <t>Competence_Register_v2.0_Template.xlsx</t>
-        </is>
-      </c>
-      <c r="N39" s="13" t="inlineStr">
-        <is>
-          <t>Compliance Monitoring Pack; Senior Management Pack</t>
-        </is>
-      </c>
+          <t>Fair_Value_Register_v2.0_Template.xlsx</t>
+        </is>
+      </c>
+      <c r="N39" s="13" t="n"/>
     </row>
     <row r="40">
       <c r="B40" s="13" t="inlineStr">
         <is>
-          <t>CPD Log</t>
+          <t>Consumer Duty Board Report Actions</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>Training Pack</t>
+          <t>Consumer Duty Pack</t>
         </is>
       </c>
       <c r="D40" s="13" t="n"/>
@@ -2227,7 +2203,7 @@
       </c>
       <c r="M40" s="13" t="inlineStr">
         <is>
-          <t>CPD_Log_v2.0_Template.xlsx</t>
+          <t>Consumer_Duty_Board_Report_Actions_v2.0_Template.xlsx</t>
         </is>
       </c>
       <c r="N40" s="13" t="n"/>
@@ -2235,12 +2211,12 @@
     <row r="41">
       <c r="B41" s="13" t="inlineStr">
         <is>
-          <t>Individual Training Record (optional)</t>
+          <t>Financial Promotions Policy</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
         <is>
-          <t>Training Pack</t>
+          <t>Consumer Duty Pack</t>
         </is>
       </c>
       <c r="D41" s="13" t="n"/>
@@ -2265,12 +2241,12 @@
       </c>
       <c r="L41" s="13" t="inlineStr">
         <is>
-          <t>Register.</t>
+          <t>Policy.</t>
         </is>
       </c>
       <c r="M41" s="13" t="inlineStr">
         <is>
-          <t>Individual_Training_Record_v2.0_Template.xlsx</t>
+          <t>Financial_Promotions_Policy_v2.0_Template.docx</t>
         </is>
       </c>
       <c r="N41" s="13" t="n"/>
@@ -2278,24 +2254,16 @@
     <row r="42">
       <c r="B42" s="13" t="inlineStr">
         <is>
-          <t>Data Processing Policy</t>
+          <t>Financial Promotions Log</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>Data Protection Pack</t>
-        </is>
-      </c>
-      <c r="D42" s="19" t="inlineStr">
-        <is>
-          <t>[Set price]</t>
-        </is>
-      </c>
-      <c r="E42" s="19" t="inlineStr">
-        <is>
-          <t>[Create Payment Link in Stripe]</t>
-        </is>
-      </c>
+          <t>Consumer Duty Pack</t>
+        </is>
+      </c>
+      <c r="D42" s="13" t="n"/>
+      <c r="E42" s="13" t="n"/>
       <c r="F42" s="13" t="n"/>
       <c r="G42" s="13" t="inlineStr">
         <is>
@@ -2316,25 +2284,29 @@
       </c>
       <c r="L42" s="13" t="inlineStr">
         <is>
-          <t>Policy. NEW PACK – set price and create a Stripe Payment Link (with package_id metadata) before selling.</t>
+          <t>Register.</t>
         </is>
       </c>
       <c r="M42" s="13" t="inlineStr">
         <is>
-          <t>Data_Processing_Policy_v2.0_Template.docx</t>
-        </is>
-      </c>
-      <c r="N42" s="13" t="n"/>
+          <t>Financial_Promotions_Log_v2.0_Template.xlsx</t>
+        </is>
+      </c>
+      <c r="N42" s="13" t="inlineStr">
+        <is>
+          <t>Compliance Monitoring Pack</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="B43" s="13" t="inlineStr">
         <is>
-          <t>Record of Processing Activities</t>
+          <t>Financial Promotion Approval Checklist</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
         <is>
-          <t>Data Protection Pack</t>
+          <t>Consumer Duty Pack</t>
         </is>
       </c>
       <c r="D43" s="13" t="n"/>
@@ -2364,28 +2336,30 @@
       </c>
       <c r="M43" s="13" t="inlineStr">
         <is>
-          <t>Record_of_Processing_Activities_v2.0_Template.xlsx</t>
-        </is>
-      </c>
-      <c r="N43" s="13" t="inlineStr">
-        <is>
-          <t>Customer Due Diligence Pack</t>
-        </is>
-      </c>
+          <t>Financial_Promotion_Approval_Checklist_v2.0_Template.xlsx</t>
+        </is>
+      </c>
+      <c r="N43" s="13" t="n"/>
     </row>
     <row r="44">
       <c r="B44" s="13" t="inlineStr">
         <is>
-          <t>Data Rights Request Log</t>
+          <t>Risk Management Framework</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>Data Protection Pack</t>
-        </is>
-      </c>
-      <c r="D44" s="13" t="n"/>
-      <c r="E44" s="13" t="n"/>
+          <t>Risk Management Pack</t>
+        </is>
+      </c>
+      <c r="D44" s="14" t="n">
+        <v>35</v>
+      </c>
+      <c r="E44" s="18" t="inlineStr">
+        <is>
+          <t>https://buy.stripe.com/7sY14g9xb5tz8Wl41Zfbq07</t>
+        </is>
+      </c>
       <c r="F44" s="13" t="n"/>
       <c r="G44" s="13" t="inlineStr">
         <is>
@@ -2406,29 +2380,25 @@
       </c>
       <c r="L44" s="13" t="inlineStr">
         <is>
-          <t>Register.</t>
+          <t>Policy.</t>
         </is>
       </c>
       <c r="M44" s="13" t="inlineStr">
         <is>
-          <t>Data_Rights_Request_Log_v2.0_Template.xlsx</t>
-        </is>
-      </c>
-      <c r="N44" s="13" t="inlineStr">
-        <is>
-          <t>Compliance Monitoring Pack</t>
-        </is>
-      </c>
+          <t>Risk_Management_Framework_v2.0_Template.docx</t>
+        </is>
+      </c>
+      <c r="N44" s="13" t="n"/>
     </row>
     <row r="45">
       <c r="B45" s="13" t="inlineStr">
         <is>
-          <t>Data Breach Log</t>
+          <t>Risk Assessment Log</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
         <is>
-          <t>Data Protection Pack</t>
+          <t>Risk Management Pack</t>
         </is>
       </c>
       <c r="D45" s="13" t="n"/>
@@ -2458,28 +2428,34 @@
       </c>
       <c r="M45" s="13" t="inlineStr">
         <is>
-          <t>Data_Breach_Log_v2.0_Template.xlsx</t>
+          <t>Risk_Assessment_Log_v2.0_Template.xlsx</t>
         </is>
       </c>
       <c r="N45" s="13" t="inlineStr">
         <is>
-          <t>Compliance Monitoring Pack</t>
+          <t>Compliance Monitoring Pack; Consumer Duty Pack</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="13" t="inlineStr">
         <is>
-          <t>Data Protection Complaints Log</t>
+          <t>Training and Competence Policy</t>
         </is>
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>Data Protection Pack</t>
-        </is>
-      </c>
-      <c r="D46" s="13" t="n"/>
-      <c r="E46" s="13" t="n"/>
+          <t>Training Pack</t>
+        </is>
+      </c>
+      <c r="D46" s="14" t="n">
+        <v>25</v>
+      </c>
+      <c r="E46" s="18" t="inlineStr">
+        <is>
+          <t>https://buy.stripe.com/eVq28kaBf09fa0p6a7fbq08</t>
+        </is>
+      </c>
       <c r="F46" s="13" t="n"/>
       <c r="G46" s="13" t="inlineStr">
         <is>
@@ -2500,29 +2476,25 @@
       </c>
       <c r="L46" s="13" t="inlineStr">
         <is>
-          <t>Register.</t>
+          <t>Policy.</t>
         </is>
       </c>
       <c r="M46" s="13" t="inlineStr">
         <is>
-          <t>Data_Protection_Complaints_Log_v2.0_Template.xlsx</t>
-        </is>
-      </c>
-      <c r="N46" s="13" t="inlineStr">
-        <is>
-          <t>Complaints Pack</t>
-        </is>
-      </c>
+          <t>Training_and_Competence_Policy_v2.0_Template.docx</t>
+        </is>
+      </c>
+      <c r="N46" s="13" t="n"/>
     </row>
     <row r="47">
       <c r="B47" s="13" t="inlineStr">
         <is>
-          <t>Data Retention Schedule</t>
+          <t>Training Matrix</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
         <is>
-          <t>Data Protection Pack</t>
+          <t>Training Pack</t>
         </is>
       </c>
       <c r="D47" s="13" t="n"/>
@@ -2552,7 +2524,7 @@
       </c>
       <c r="M47" s="13" t="inlineStr">
         <is>
-          <t>Data_Retention_Schedule_v2.0_Template.xlsx</t>
+          <t>Training_Matrix_v2.0_Template.xlsx</t>
         </is>
       </c>
       <c r="N47" s="13" t="n"/>
@@ -2560,12 +2532,12 @@
     <row r="48">
       <c r="B48" s="13" t="inlineStr">
         <is>
-          <t>DPIA Register</t>
+          <t>Training Log</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
         <is>
-          <t>Data Protection Pack</t>
+          <t>Training Pack</t>
         </is>
       </c>
       <c r="D48" s="13" t="n"/>
@@ -2595,32 +2567,28 @@
       </c>
       <c r="M48" s="13" t="inlineStr">
         <is>
-          <t>DPIA_Register_v2.0_Template.xlsx</t>
-        </is>
-      </c>
-      <c r="N48" s="13" t="n"/>
+          <t>Training_Log_v2.0_Template.xlsx</t>
+        </is>
+      </c>
+      <c r="N48" s="13" t="inlineStr">
+        <is>
+          <t>All other packs</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="B49" s="13" t="inlineStr">
         <is>
-          <t>Financial Promotions Policy</t>
+          <t>Competence Register</t>
         </is>
       </c>
       <c r="C49" s="13" t="inlineStr">
         <is>
-          <t>Financial Promotions Pack</t>
-        </is>
-      </c>
-      <c r="D49" s="19" t="inlineStr">
-        <is>
-          <t>[Set price]</t>
-        </is>
-      </c>
-      <c r="E49" s="19" t="inlineStr">
-        <is>
-          <t>[Create Payment Link in Stripe]</t>
-        </is>
-      </c>
+          <t>Training Pack</t>
+        </is>
+      </c>
+      <c r="D49" s="13" t="n"/>
+      <c r="E49" s="13" t="n"/>
       <c r="F49" s="13" t="n"/>
       <c r="G49" s="13" t="inlineStr">
         <is>
@@ -2641,25 +2609,29 @@
       </c>
       <c r="L49" s="13" t="inlineStr">
         <is>
-          <t>Policy. NEW PACK – set price and create a Stripe Payment Link (with package_id metadata) before selling.</t>
+          <t>Register.</t>
         </is>
       </c>
       <c r="M49" s="13" t="inlineStr">
         <is>
-          <t>Financial_Promotions_Policy_v2.0_Template.docx</t>
-        </is>
-      </c>
-      <c r="N49" s="13" t="n"/>
+          <t>Competence_Register_v2.0_Template.xlsx</t>
+        </is>
+      </c>
+      <c r="N49" s="13" t="inlineStr">
+        <is>
+          <t>Compliance Monitoring Pack; Senior Management Pack</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="B50" s="13" t="inlineStr">
         <is>
-          <t>Financial Promotions Log</t>
+          <t>CPD Log</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
         <is>
-          <t>Financial Promotions Pack</t>
+          <t>Training Pack</t>
         </is>
       </c>
       <c r="D50" s="13" t="n"/>
@@ -2689,24 +2661,20 @@
       </c>
       <c r="M50" s="13" t="inlineStr">
         <is>
-          <t>Financial_Promotions_Log_v2.0_Template.xlsx</t>
-        </is>
-      </c>
-      <c r="N50" s="13" t="inlineStr">
-        <is>
-          <t>Compliance Monitoring Pack</t>
-        </is>
-      </c>
+          <t>CPD_Log_v2.0_Template.xlsx</t>
+        </is>
+      </c>
+      <c r="N50" s="13" t="n"/>
     </row>
     <row r="51">
       <c r="B51" s="13" t="inlineStr">
         <is>
-          <t>Financial Promotion Approval Checklist</t>
+          <t>Individual Training Record (optional)</t>
         </is>
       </c>
       <c r="C51" s="13" t="inlineStr">
         <is>
-          <t>Financial Promotions Pack</t>
+          <t>Training Pack</t>
         </is>
       </c>
       <c r="D51" s="13" t="n"/>
@@ -2736,47 +2704,47 @@
       </c>
       <c r="M51" s="13" t="inlineStr">
         <is>
-          <t>Financial_Promotion_Approval_Checklist_v2.0_Template.xlsx</t>
+          <t>Individual_Training_Record_v2.0_Template.xlsx</t>
         </is>
       </c>
       <c r="N51" s="13" t="n"/>
     </row>
     <row r="52">
-      <c r="B52" s="20" t="inlineStr">
+      <c r="B52" s="19" t="inlineStr">
         <is>
           <t>Complete Authorisation Pack</t>
         </is>
       </c>
-      <c r="C52" s="21" t="inlineStr">
+      <c r="C52" s="20" t="inlineStr">
         <is>
           <t>Complete Authorisation Pack</t>
         </is>
       </c>
-      <c r="D52" s="22" t="n">
+      <c r="D52" s="21" t="n">
         <v>200</v>
       </c>
-      <c r="E52" s="23" t="inlineStr">
+      <c r="E52" s="22" t="inlineStr">
         <is>
           <t>https://buy.stripe.com/6oUcMY38NaNT7Shaqnfbq03</t>
         </is>
       </c>
-      <c r="F52" s="21" t="n"/>
-      <c r="G52" s="21" t="n"/>
-      <c r="H52" s="21" t="n"/>
-      <c r="I52" s="21" t="n"/>
-      <c r="J52" s="21" t="n"/>
-      <c r="K52" s="21" t="n"/>
-      <c r="L52" s="21" t="inlineStr">
-        <is>
-          <t>Bundle of every document above (45 files: 12 policies, 32 registers and the FIT and Proper Questionnaire). Price unchanged – check the “save £50 vs £250” wording on the website now that two new packs exist.</t>
-        </is>
-      </c>
-      <c r="M52" s="21" t="inlineStr">
+      <c r="F52" s="20" t="n"/>
+      <c r="G52" s="20" t="n"/>
+      <c r="H52" s="20" t="n"/>
+      <c r="I52" s="20" t="n"/>
+      <c r="J52" s="20" t="n"/>
+      <c r="K52" s="20" t="n"/>
+      <c r="L52" s="20" t="inlineStr">
+        <is>
+          <t>Bundle of every document above (45 files: 12 policies, 32 registers and the FIT and Proper Questionnaire). Price unchanged. The eight individual packs still total £250, so the website’s “save £50” wording remains correct.</t>
+        </is>
+      </c>
+      <c r="M52" s="20" t="inlineStr">
         <is>
           <t>All files listed above</t>
         </is>
       </c>
-      <c r="N52" s="21" t="n"/>
+      <c r="N52" s="20" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="B6:N52">
@@ -2791,11 +2759,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Remove shared-register column: each register ships with its main pack only
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0185GJD35Lj4maZQfYQD6Tsw
</commit_message>
<xml_diff>
--- a/framework-templates/Document_Log_Pricing_v2.0.xlsx
+++ b/framework-templates/Document_Log_Pricing_v2.0.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Document Log" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Document Log'!$B$6:$N$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Document Log'!$B$6:$M$52</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -656,11 +656,6 @@
           <t>File Name</t>
         </is>
       </c>
-      <c r="N6" s="3" t="inlineStr">
-        <is>
-          <t>Also Supplied In (register required by these packs’ policies)</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="B7" s="13" t="inlineStr">
@@ -709,7 +704,6 @@
           <t>Anti_Money_Laundering_Policy_v2.0_Template.docx</t>
         </is>
       </c>
-      <c r="N7" s="13" t="n"/>
     </row>
     <row r="8">
       <c r="B8" s="13" t="inlineStr">
@@ -752,7 +746,6 @@
           <t>Anti_Money_Laundering_Incident_Register_v2.0_Template.docx</t>
         </is>
       </c>
-      <c r="N8" s="13" t="n"/>
     </row>
     <row r="9">
       <c r="B9" s="13" t="inlineStr">
@@ -795,11 +788,6 @@
           <t>AML_Business_Wide_Risk_Assessment_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N9" s="13" t="inlineStr">
-        <is>
-          <t>Risk Management Pack; Customer Due Diligence Pack</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="B10" s="13" t="inlineStr">
@@ -842,11 +830,6 @@
           <t>Sanctions_Screening_Log_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N10" s="13" t="inlineStr">
-        <is>
-          <t>Customer Due Diligence Pack; Compliance Monitoring Pack</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="B11" s="13" t="inlineStr">
@@ -889,11 +872,6 @@
           <t>Conflicts_of_Interest_Register_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N11" s="13" t="inlineStr">
-        <is>
-          <t>Compliance Monitoring Pack</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="B12" s="13" t="inlineStr">
@@ -936,11 +914,6 @@
           <t>Gifts_and_Hospitality_Register_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N12" s="13" t="inlineStr">
-        <is>
-          <t>Compliance Monitoring Pack</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="B13" s="13" t="inlineStr">
@@ -989,7 +962,6 @@
           <t>Complaints_Procedure_v2.0_Template.docx</t>
         </is>
       </c>
-      <c r="N13" s="13" t="n"/>
     </row>
     <row r="14">
       <c r="B14" s="13" t="inlineStr">
@@ -1032,11 +1004,6 @@
           <t>Complaints_Register_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N14" s="13" t="inlineStr">
-        <is>
-          <t>Compliance Monitoring Pack; Customer Due Diligence Pack; Consumer Duty Pack</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="B15" s="13" t="inlineStr">
@@ -1079,11 +1046,6 @@
           <t>Compliance_Breach_Log_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N15" s="13" t="inlineStr">
-        <is>
-          <t>AML Pack; Compliance Monitoring Pack; Risk Management Pack; Training Pack</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="B16" s="13" t="inlineStr">
@@ -1132,7 +1094,6 @@
           <t>Compliance_Monitoring_Plan_v2.0_Template.docx</t>
         </is>
       </c>
-      <c r="N16" s="13" t="n"/>
     </row>
     <row r="17">
       <c r="B17" s="13" t="inlineStr">
@@ -1175,7 +1136,6 @@
           <t>Compliance_Monitoring_Programme_Policy_v2.0_Template.docx</t>
         </is>
       </c>
-      <c r="N17" s="13" t="n"/>
     </row>
     <row r="18">
       <c r="B18" s="13" t="inlineStr">
@@ -1218,11 +1178,6 @@
           <t>Compliance_Monitoring_Schedule_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N18" s="13" t="inlineStr">
-        <is>
-          <t>Training Pack; Consumer Duty Pack</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="B19" s="13" t="inlineStr">
@@ -1265,7 +1220,6 @@
           <t>File_Review_Record_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N19" s="13" t="n"/>
     </row>
     <row r="20">
       <c r="B20" s="13" t="inlineStr">
@@ -1308,11 +1262,6 @@
           <t>Corrective_Action_Log_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N20" s="13" t="inlineStr">
-        <is>
-          <t>Complaints Pack; Risk Management Pack</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="B21" s="13" t="inlineStr">
@@ -1355,7 +1304,6 @@
           <t>Compliance_Universe_Register_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N21" s="13" t="n"/>
     </row>
     <row r="22">
       <c r="B22" s="13" t="inlineStr">
@@ -1398,7 +1346,6 @@
           <t>Data_Processing_Policy_v2.0_Template.docx</t>
         </is>
       </c>
-      <c r="N22" s="13" t="n"/>
     </row>
     <row r="23">
       <c r="B23" s="13" t="inlineStr">
@@ -1441,11 +1388,6 @@
           <t>Record_of_Processing_Activities_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N23" s="13" t="inlineStr">
-        <is>
-          <t>Customer Due Diligence Pack</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="B24" s="13" t="inlineStr">
@@ -1488,7 +1430,6 @@
           <t>Data_Rights_Request_Log_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N24" s="13" t="n"/>
     </row>
     <row r="25">
       <c r="B25" s="13" t="inlineStr">
@@ -1531,7 +1472,6 @@
           <t>Data_Breach_Log_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N25" s="13" t="n"/>
     </row>
     <row r="26">
       <c r="B26" s="13" t="inlineStr">
@@ -1574,11 +1514,6 @@
           <t>Data_Protection_Complaints_Log_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N26" s="13" t="inlineStr">
-        <is>
-          <t>Complaints Pack</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="B27" s="13" t="inlineStr">
@@ -1621,7 +1556,6 @@
           <t>Data_Retention_Schedule_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N27" s="13" t="n"/>
     </row>
     <row r="28">
       <c r="B28" s="13" t="inlineStr">
@@ -1664,7 +1598,6 @@
           <t>DPIA_Register_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N28" s="13" t="n"/>
     </row>
     <row r="29">
       <c r="B29" s="13" t="inlineStr">
@@ -1713,7 +1646,6 @@
           <t>Customer_Due_Diligence_Policy_v2.0_Template.docx</t>
         </is>
       </c>
-      <c r="N29" s="13" t="n"/>
     </row>
     <row r="30">
       <c r="B30" s="13" t="inlineStr">
@@ -1756,7 +1688,6 @@
           <t>Customer_Vulnerability_Policy_v2.0_Template.docx</t>
         </is>
       </c>
-      <c r="N30" s="13" t="n"/>
     </row>
     <row r="31">
       <c r="B31" s="13" t="inlineStr">
@@ -1799,11 +1730,6 @@
           <t>Customer_Due_Diligence_Checklist_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N31" s="13" t="inlineStr">
-        <is>
-          <t>AML Pack</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="B32" s="13" t="inlineStr">
@@ -1846,11 +1772,6 @@
           <t>Enhanced_Due_Diligence_Checklist_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N32" s="13" t="inlineStr">
-        <is>
-          <t>AML Pack</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="B33" s="13" t="inlineStr">
@@ -1893,11 +1814,6 @@
           <t>Customer_Due_Diligence_Register_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N33" s="13" t="inlineStr">
-        <is>
-          <t>AML Pack; Compliance Monitoring Pack</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="B34" s="13" t="inlineStr">
@@ -1946,7 +1862,6 @@
           <t>SMCR_Statement_of_Responsibilities_v2.0_Template.docx</t>
         </is>
       </c>
-      <c r="N34" s="13" t="n"/>
     </row>
     <row r="35">
       <c r="B35" s="13" t="inlineStr">
@@ -1981,7 +1896,6 @@
           <t>FIT_and_Proper_Questionnaire_v1.0.docx</t>
         </is>
       </c>
-      <c r="N35" s="13" t="n"/>
     </row>
     <row r="36">
       <c r="B36" s="13" t="inlineStr">
@@ -2030,7 +1944,6 @@
           <t>Consumer_Duty_Implementation_Plan_v2.0_Template.docx</t>
         </is>
       </c>
-      <c r="N36" s="13" t="n"/>
     </row>
     <row r="37">
       <c r="B37" s="13" t="inlineStr">
@@ -2073,11 +1986,6 @@
           <t>Consumer_Duty_Outcome_MI_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N37" s="13" t="inlineStr">
-        <is>
-          <t>Complaints Pack; Compliance Monitoring Pack; Customer Due Diligence Pack; Risk Management Pack</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="B38" s="13" t="inlineStr">
@@ -2120,7 +2028,6 @@
           <t>Target_Market_Register_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N38" s="13" t="n"/>
     </row>
     <row r="39">
       <c r="B39" s="13" t="inlineStr">
@@ -2163,7 +2070,6 @@
           <t>Fair_Value_Register_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N39" s="13" t="n"/>
     </row>
     <row r="40">
       <c r="B40" s="13" t="inlineStr">
@@ -2206,7 +2112,6 @@
           <t>Consumer_Duty_Board_Report_Actions_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N40" s="13" t="n"/>
     </row>
     <row r="41">
       <c r="B41" s="13" t="inlineStr">
@@ -2249,7 +2154,6 @@
           <t>Financial_Promotions_Policy_v2.0_Template.docx</t>
         </is>
       </c>
-      <c r="N41" s="13" t="n"/>
     </row>
     <row r="42">
       <c r="B42" s="13" t="inlineStr">
@@ -2292,11 +2196,6 @@
           <t>Financial_Promotions_Log_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N42" s="13" t="inlineStr">
-        <is>
-          <t>Compliance Monitoring Pack</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="B43" s="13" t="inlineStr">
@@ -2339,7 +2238,6 @@
           <t>Financial_Promotion_Approval_Checklist_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N43" s="13" t="n"/>
     </row>
     <row r="44">
       <c r="B44" s="13" t="inlineStr">
@@ -2388,7 +2286,6 @@
           <t>Risk_Management_Framework_v2.0_Template.docx</t>
         </is>
       </c>
-      <c r="N44" s="13" t="n"/>
     </row>
     <row r="45">
       <c r="B45" s="13" t="inlineStr">
@@ -2431,11 +2328,6 @@
           <t>Risk_Assessment_Log_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N45" s="13" t="inlineStr">
-        <is>
-          <t>Compliance Monitoring Pack; Consumer Duty Pack</t>
-        </is>
-      </c>
     </row>
     <row r="46">
       <c r="B46" s="13" t="inlineStr">
@@ -2484,7 +2376,6 @@
           <t>Training_and_Competence_Policy_v2.0_Template.docx</t>
         </is>
       </c>
-      <c r="N46" s="13" t="n"/>
     </row>
     <row r="47">
       <c r="B47" s="13" t="inlineStr">
@@ -2527,7 +2418,6 @@
           <t>Training_Matrix_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N47" s="13" t="n"/>
     </row>
     <row r="48">
       <c r="B48" s="13" t="inlineStr">
@@ -2570,11 +2460,6 @@
           <t>Training_Log_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N48" s="13" t="inlineStr">
-        <is>
-          <t>All other packs</t>
-        </is>
-      </c>
     </row>
     <row r="49">
       <c r="B49" s="13" t="inlineStr">
@@ -2617,11 +2502,6 @@
           <t>Competence_Register_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N49" s="13" t="inlineStr">
-        <is>
-          <t>Compliance Monitoring Pack; Senior Management Pack</t>
-        </is>
-      </c>
     </row>
     <row r="50">
       <c r="B50" s="13" t="inlineStr">
@@ -2664,7 +2544,6 @@
           <t>CPD_Log_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N50" s="13" t="n"/>
     </row>
     <row r="51">
       <c r="B51" s="13" t="inlineStr">
@@ -2707,7 +2586,6 @@
           <t>Individual_Training_Record_v2.0_Template.xlsx</t>
         </is>
       </c>
-      <c r="N51" s="13" t="n"/>
     </row>
     <row r="52">
       <c r="B52" s="19" t="inlineStr">
@@ -2744,10 +2622,9 @@
           <t>All files listed above</t>
         </is>
       </c>
-      <c r="N52" s="20" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="B6:N52">
+  <autoFilter ref="B6:M52">
     <sortState ref="B7:L22">
       <sortCondition ref="B6:B22"/>
     </sortState>

</xml_diff>